<commit_message>
feat(spec): skill taxonomy seed file, and the alias conventions it shows
Adds public/docs/skill-taxonomy-seed.csv — 47 skills across 7 groups, each
row carrying its aliases, so the "React / ReactJS / React.js are ONE row"
rule is demonstrated rather than described. It is served from public/, so
the link in the spec resolves.

Corrects the row count in the Skill (taxonomy) note: the spec said 46, the
file has 47. A number a reader can check has to be right, or the rest of
the table stops being trusted.

Also: resume, application and jobseeker spec updates, and mockup work.
</commit_message>
<xml_diff>
--- a/Saramin_VN_CV_field_list.xlsx
+++ b/Saramin_VN_CV_field_list.xlsx
@@ -1192,7 +1192,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1565,7 +1565,7 @@
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>Highlight projects[]</t>
+          <t>Projects &amp; portfolio[]</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
@@ -1585,7 +1585,7 @@
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>Name · role · description · link.</t>
+          <t>Name · role · description · link. Also holds published papers and articles — there is no separate Publications section.</t>
         </is>
       </c>
     </row>
@@ -1642,7 +1642,7 @@
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>Publications[]</t>
+          <t>References[]</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
@@ -1663,48 +1663,52 @@
       <c r="E21" s="7" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t>References[]</t>
-        </is>
-      </c>
-      <c r="B22" s="7" t="inlineStr">
-        <is>
-          <t>repeatable</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="D22" s="7" t="inlineStr">
-        <is>
-          <t>Create</t>
-        </is>
-      </c>
-      <c r="E22" s="7" t="n"/>
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>— System / derived</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="n"/>
+      <c r="C22" s="10" t="n"/>
+      <c r="D22" s="10" t="n"/>
+      <c r="E22" s="10" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="9" t="inlineStr">
-        <is>
-          <t>— System / derived</t>
-        </is>
-      </c>
-      <c r="B23" s="10" t="n"/>
-      <c r="C23" s="10" t="n"/>
-      <c r="D23" s="10" t="n"/>
-      <c r="E23" s="10" t="n"/>
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>Completeness score</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>derived %</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>Drives the CV-completeness meter and search ranking.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>Completeness score</t>
+          <t>Field source / confidence</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>derived %</t>
+          <t>enum / 0–1</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
@@ -1719,19 +1723,19 @@
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>Drives the CV-completeness meter and search ranking.</t>
+          <t>Per field: typed by the user vs extracted by AI, and how confident the parse was.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>Field source / confidence</t>
+          <t>Created / updated at</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>enum / 0–1</t>
+          <t>timestamp</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
@@ -1745,33 +1749,6 @@
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
-        <is>
-          <t>Per field: typed by the user vs extracted by AI, and how confident the parse was.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="7" t="inlineStr">
-        <is>
-          <t>Created / updated at</t>
-        </is>
-      </c>
-      <c r="B26" s="7" t="inlineStr">
-        <is>
-          <t>timestamp</t>
-        </is>
-      </c>
-      <c r="C26" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D26" s="7" t="inlineStr">
-        <is>
-          <t>System</t>
-        </is>
-      </c>
-      <c r="E26" s="7" t="inlineStr">
         <is>
           <t>Recency is a search-ranking signal.</t>
         </is>

</xml_diff>